<commit_message>
Found a new data source for Georgia. Only West Virginia and New Mexico remain unverified.
</commit_message>
<xml_diff>
--- a/data/raw/State_Sources.xlsx
+++ b/data/raw/State_Sources.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chigham\Documents\forkranger-us-regions\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEBAA7B4-22EB-437B-B6A2-2C5DFCE931BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE2235EC-A946-43A7-9500-90553C2C30C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34365" yWindow="2970" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{1A035CB0-260D-4ABF-9F3B-5033D39FF1A0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{1A035CB0-260D-4ABF-9F3B-5033D39FF1A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Alabama" sheetId="1" r:id="rId1"/>
@@ -93,8 +93,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={B356F055-D067-4C15-8726-A70F0593CFCD}</author>
+  </authors>
+  <commentList>
+    <comment ref="A20" authorId="0" shapeId="0" xr:uid="{B356F055-D067-4C15-8726-A70F0593CFCD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Consider adding this one</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14939" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15179" uniqueCount="533">
   <si>
     <t>Greens (Collards, turnips, etc.)</t>
   </si>
@@ -1623,9 +1641,6 @@
     <t>Not Applicable</t>
   </si>
   <si>
-    <t>Merge? Peas?</t>
-  </si>
-  <si>
     <t>Bell pepper</t>
   </si>
   <si>
@@ -1641,22 +1656,13 @@
     <t>Cherry</t>
   </si>
   <si>
-    <t>Merge? Melons?</t>
-  </si>
-  <si>
     <t>Rocket</t>
   </si>
   <si>
     <t>Red cabbage</t>
   </si>
   <si>
-    <t>Merge? Bell Peppers?</t>
-  </si>
-  <si>
     <t>White cabbage</t>
-  </si>
-  <si>
-    <t>Merge? Potato?</t>
   </si>
   <si>
     <t>Savoy cabbage</t>
@@ -1672,6 +1678,39 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Consider Adding</t>
+  </si>
+  <si>
+    <t>Add</t>
+  </si>
+  <si>
+    <t>Add (includes Butternut)</t>
+  </si>
+  <si>
+    <t>Watermelon ??</t>
+  </si>
+  <si>
+    <t>Pakchoi ? Add</t>
+  </si>
+  <si>
+    <t>Merge? Melons? Keep separate for now</t>
+  </si>
+  <si>
+    <t>Merge? Bell Peppers? Keep separate for now</t>
+  </si>
+  <si>
+    <t>Merge? Potato? Keep separate for now</t>
+  </si>
+  <si>
+    <t>Consider adding</t>
+  </si>
+  <si>
+    <t>https://www.gfb.org/learn/georgia-neighbors/post/georgia-harvest-calendar</t>
+  </si>
+  <si>
+    <t>Extended Season</t>
   </si>
 </sst>
 </file>
@@ -1707,38 +1746,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="5">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1792,20 +1805,20 @@
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1822,6 +1835,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Higham, Christopher A. (LARC-E302)[BOOZ ALLEN HAMILTON INC]" id="{72AD52FB-2964-4D77-8D4D-94C656643D63}" userId="S::chigham@ndc.nasa.gov::13092c3f-58b6-42cd-a241-9fd72d0b9084" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2139,13 +2158,22 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A20" dT="2025-10-17T12:20:39.70" personId="{72AD52FB-2964-4D77-8D4D-94C656643D63}" id="{B356F055-D067-4C15-8726-A70F0593CFCD}">
+    <text>Consider adding this one</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12941840-B272-4527-BC1E-49BD698D2692}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12941840-B272-4527-BC1E-49BD698D2692}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:O37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="27.6640625" customWidth="1"/>
+    <col min="1" max="1" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" customWidth="1"/>
     <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="12" width="11.77734375" bestFit="1" customWidth="1"/>
     <col min="13" max="14" width="11.21875" bestFit="1" customWidth="1"/>
@@ -2335,7 +2363,7 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="F8" t="s">
         <v>238</v>
@@ -2538,7 +2566,7 @@
       <c r="A17" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C17" t="s">
@@ -2650,7 +2678,7 @@
         <v>27</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>508</v>
+        <v>522</v>
       </c>
       <c r="H20" t="s">
         <v>238</v>
@@ -2724,11 +2752,11 @@
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
+      <c r="A23" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="5" t="s">
-        <v>509</v>
+      <c r="B23" t="s">
+        <v>45</v>
       </c>
       <c r="F23" t="s">
         <v>238</v>
@@ -2744,10 +2772,12 @@
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
+      <c r="A24" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="6"/>
+      <c r="B24" s="1" t="s">
+        <v>508</v>
+      </c>
       <c r="G24" t="s">
         <v>238</v>
       </c>
@@ -2795,7 +2825,7 @@
         <v>22</v>
       </c>
       <c r="B26" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H26" t="s">
         <v>238</v>
@@ -3079,11 +3109,9 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O37">
     <sortCondition ref="A2:A37"/>
   </sortState>
-  <mergeCells count="1">
-    <mergeCell ref="B23:B24"/>
-  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4608,10 +4636,16 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA85BFD1-C222-47FB-A597-3386D423A900}">
   <sheetPr codeName="Sheet11"/>
-  <dimension ref="B1:M1"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="9" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="12" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -4647,6 +4681,780 @@
       </c>
       <c r="M1" t="s">
         <v>251</v>
+      </c>
+      <c r="N1" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" t="s">
+        <v>238</v>
+      </c>
+      <c r="I2" t="s">
+        <v>239</v>
+      </c>
+      <c r="J2" t="s">
+        <v>239</v>
+      </c>
+      <c r="K2" t="s">
+        <v>239</v>
+      </c>
+      <c r="L2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" t="s">
+        <v>238</v>
+      </c>
+      <c r="G3" t="s">
+        <v>239</v>
+      </c>
+      <c r="H3" t="s">
+        <v>239</v>
+      </c>
+      <c r="I3" t="s">
+        <v>239</v>
+      </c>
+      <c r="J3" t="s">
+        <v>239</v>
+      </c>
+      <c r="K3" t="s">
+        <v>239</v>
+      </c>
+      <c r="L3" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>238</v>
+      </c>
+      <c r="G4" t="s">
+        <v>239</v>
+      </c>
+      <c r="H4" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>238</v>
+      </c>
+      <c r="G5" t="s">
+        <v>239</v>
+      </c>
+      <c r="H5" t="s">
+        <v>239</v>
+      </c>
+      <c r="I5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" t="s">
+        <v>238</v>
+      </c>
+      <c r="G6" t="s">
+        <v>237</v>
+      </c>
+      <c r="K6" t="s">
+        <v>238</v>
+      </c>
+      <c r="L6" t="s">
+        <v>239</v>
+      </c>
+      <c r="M6" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" t="s">
+        <v>239</v>
+      </c>
+      <c r="C7" t="s">
+        <v>237</v>
+      </c>
+      <c r="L7" t="s">
+        <v>238</v>
+      </c>
+      <c r="M7" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>239</v>
+      </c>
+      <c r="C8" t="s">
+        <v>239</v>
+      </c>
+      <c r="D8" t="s">
+        <v>239</v>
+      </c>
+      <c r="E8" t="s">
+        <v>239</v>
+      </c>
+      <c r="F8" t="s">
+        <v>237</v>
+      </c>
+      <c r="K8" t="s">
+        <v>238</v>
+      </c>
+      <c r="L8" t="s">
+        <v>239</v>
+      </c>
+      <c r="M8" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" t="s">
+        <v>238</v>
+      </c>
+      <c r="H9" t="s">
+        <v>239</v>
+      </c>
+      <c r="I9" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" t="s">
+        <v>239</v>
+      </c>
+      <c r="C10" t="s">
+        <v>239</v>
+      </c>
+      <c r="D10" t="s">
+        <v>239</v>
+      </c>
+      <c r="E10" t="s">
+        <v>239</v>
+      </c>
+      <c r="F10" t="s">
+        <v>237</v>
+      </c>
+      <c r="K10" t="s">
+        <v>238</v>
+      </c>
+      <c r="L10" t="s">
+        <v>239</v>
+      </c>
+      <c r="M10" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" t="s">
+        <v>239</v>
+      </c>
+      <c r="C11" t="s">
+        <v>239</v>
+      </c>
+      <c r="D11" t="s">
+        <v>237</v>
+      </c>
+      <c r="J11" t="s">
+        <v>238</v>
+      </c>
+      <c r="K11" t="s">
+        <v>239</v>
+      </c>
+      <c r="L11" t="s">
+        <v>239</v>
+      </c>
+      <c r="M11" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>230</v>
+      </c>
+      <c r="B12" t="s">
+        <v>239</v>
+      </c>
+      <c r="C12" t="s">
+        <v>239</v>
+      </c>
+      <c r="D12" t="s">
+        <v>239</v>
+      </c>
+      <c r="E12" t="s">
+        <v>239</v>
+      </c>
+      <c r="F12" t="s">
+        <v>239</v>
+      </c>
+      <c r="G12" t="s">
+        <v>237</v>
+      </c>
+      <c r="K12" t="s">
+        <v>238</v>
+      </c>
+      <c r="L12" t="s">
+        <v>239</v>
+      </c>
+      <c r="M12" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" t="s">
+        <v>238</v>
+      </c>
+      <c r="H13" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" t="s">
+        <v>238</v>
+      </c>
+      <c r="H14" t="s">
+        <v>239</v>
+      </c>
+      <c r="I14" t="s">
+        <v>239</v>
+      </c>
+      <c r="J14" t="s">
+        <v>532</v>
+      </c>
+      <c r="K14" t="s">
+        <v>532</v>
+      </c>
+      <c r="L14" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" t="s">
+        <v>238</v>
+      </c>
+      <c r="H15" t="s">
+        <v>239</v>
+      </c>
+      <c r="I15" t="s">
+        <v>239</v>
+      </c>
+      <c r="J15" t="s">
+        <v>239</v>
+      </c>
+      <c r="K15" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>123</v>
+      </c>
+      <c r="H16" t="s">
+        <v>238</v>
+      </c>
+      <c r="I16" t="s">
+        <v>239</v>
+      </c>
+      <c r="J16" t="s">
+        <v>239</v>
+      </c>
+      <c r="K16" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" t="s">
+        <v>532</v>
+      </c>
+      <c r="C17" t="s">
+        <v>532</v>
+      </c>
+      <c r="D17" t="s">
+        <v>239</v>
+      </c>
+      <c r="E17" t="s">
+        <v>239</v>
+      </c>
+      <c r="F17" t="s">
+        <v>237</v>
+      </c>
+      <c r="K17" t="s">
+        <v>238</v>
+      </c>
+      <c r="L17" t="s">
+        <v>239</v>
+      </c>
+      <c r="M17" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" t="s">
+        <v>532</v>
+      </c>
+      <c r="C18" t="s">
+        <v>532</v>
+      </c>
+      <c r="D18" t="s">
+        <v>239</v>
+      </c>
+      <c r="E18" t="s">
+        <v>239</v>
+      </c>
+      <c r="F18" t="s">
+        <v>239</v>
+      </c>
+      <c r="G18" t="s">
+        <v>237</v>
+      </c>
+      <c r="J18" t="s">
+        <v>238</v>
+      </c>
+      <c r="K18" t="s">
+        <v>239</v>
+      </c>
+      <c r="L18" t="s">
+        <v>239</v>
+      </c>
+      <c r="M18" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>144</v>
+      </c>
+      <c r="B19" t="s">
+        <v>239</v>
+      </c>
+      <c r="C19" t="s">
+        <v>239</v>
+      </c>
+      <c r="D19" t="s">
+        <v>239</v>
+      </c>
+      <c r="E19" t="s">
+        <v>239</v>
+      </c>
+      <c r="F19" t="s">
+        <v>239</v>
+      </c>
+      <c r="G19" t="s">
+        <v>239</v>
+      </c>
+      <c r="H19" t="s">
+        <v>239</v>
+      </c>
+      <c r="I19" t="s">
+        <v>239</v>
+      </c>
+      <c r="J19" t="s">
+        <v>239</v>
+      </c>
+      <c r="K19" t="s">
+        <v>239</v>
+      </c>
+      <c r="L19" t="s">
+        <v>239</v>
+      </c>
+      <c r="M19" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="F20" t="s">
+        <v>238</v>
+      </c>
+      <c r="G20" t="s">
+        <v>239</v>
+      </c>
+      <c r="H20" t="s">
+        <v>239</v>
+      </c>
+      <c r="I20" t="s">
+        <v>239</v>
+      </c>
+      <c r="J20" t="s">
+        <v>239</v>
+      </c>
+      <c r="K20" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" t="s">
+        <v>238</v>
+      </c>
+      <c r="F21" t="s">
+        <v>239</v>
+      </c>
+      <c r="G21" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" t="s">
+        <v>238</v>
+      </c>
+      <c r="G22" t="s">
+        <v>239</v>
+      </c>
+      <c r="H22" t="s">
+        <v>239</v>
+      </c>
+      <c r="I22" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>2</v>
+      </c>
+      <c r="J23" t="s">
+        <v>238</v>
+      </c>
+      <c r="K23" t="s">
+        <v>239</v>
+      </c>
+      <c r="L23" t="s">
+        <v>239</v>
+      </c>
+      <c r="M23" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24" t="s">
+        <v>238</v>
+      </c>
+      <c r="I24" t="s">
+        <v>239</v>
+      </c>
+      <c r="J24" t="s">
+        <v>239</v>
+      </c>
+      <c r="K24" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>158</v>
+      </c>
+      <c r="H25" t="s">
+        <v>238</v>
+      </c>
+      <c r="I25" t="s">
+        <v>239</v>
+      </c>
+      <c r="J25" t="s">
+        <v>239</v>
+      </c>
+      <c r="K25" t="s">
+        <v>239</v>
+      </c>
+      <c r="L25" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" t="s">
+        <v>238</v>
+      </c>
+      <c r="G26" t="s">
+        <v>239</v>
+      </c>
+      <c r="H26" t="s">
+        <v>239</v>
+      </c>
+      <c r="I26" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>167</v>
+      </c>
+      <c r="B27" t="s">
+        <v>239</v>
+      </c>
+      <c r="C27" t="s">
+        <v>237</v>
+      </c>
+      <c r="I27" t="s">
+        <v>238</v>
+      </c>
+      <c r="J27" t="s">
+        <v>239</v>
+      </c>
+      <c r="K27" t="s">
+        <v>239</v>
+      </c>
+      <c r="L27" t="s">
+        <v>239</v>
+      </c>
+      <c r="M27" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>33</v>
+      </c>
+      <c r="J28" t="s">
+        <v>238</v>
+      </c>
+      <c r="K28" t="s">
+        <v>239</v>
+      </c>
+      <c r="L28" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>47</v>
+      </c>
+      <c r="G29" t="s">
+        <v>238</v>
+      </c>
+      <c r="H29" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" t="s">
+        <v>239</v>
+      </c>
+      <c r="C30" t="s">
+        <v>239</v>
+      </c>
+      <c r="D30" t="s">
+        <v>239</v>
+      </c>
+      <c r="E30" t="s">
+        <v>239</v>
+      </c>
+      <c r="F30" t="s">
+        <v>237</v>
+      </c>
+      <c r="L30" t="s">
+        <v>238</v>
+      </c>
+      <c r="M30" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>161</v>
+      </c>
+      <c r="F31" t="s">
+        <v>238</v>
+      </c>
+      <c r="G31" t="s">
+        <v>239</v>
+      </c>
+      <c r="H31" t="s">
+        <v>239</v>
+      </c>
+      <c r="I31" t="s">
+        <v>239</v>
+      </c>
+      <c r="J31" t="s">
+        <v>239</v>
+      </c>
+      <c r="K31" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>50</v>
+      </c>
+      <c r="I32" t="s">
+        <v>238</v>
+      </c>
+      <c r="J32" t="s">
+        <v>239</v>
+      </c>
+      <c r="K32" t="s">
+        <v>239</v>
+      </c>
+      <c r="L32" t="s">
+        <v>239</v>
+      </c>
+      <c r="M32" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>4</v>
+      </c>
+      <c r="D33" t="s">
+        <v>238</v>
+      </c>
+      <c r="E33" t="s">
+        <v>239</v>
+      </c>
+      <c r="F33" t="s">
+        <v>239</v>
+      </c>
+      <c r="G33" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>23</v>
+      </c>
+      <c r="F34" t="s">
+        <v>238</v>
+      </c>
+      <c r="G34" t="s">
+        <v>239</v>
+      </c>
+      <c r="H34" t="s">
+        <v>239</v>
+      </c>
+      <c r="I34" t="s">
+        <v>239</v>
+      </c>
+      <c r="J34" t="s">
+        <v>239</v>
+      </c>
+      <c r="K34" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" t="s">
+        <v>532</v>
+      </c>
+      <c r="C35" t="s">
+        <v>532</v>
+      </c>
+      <c r="D35" t="s">
+        <v>239</v>
+      </c>
+      <c r="E35" t="s">
+        <v>237</v>
+      </c>
+      <c r="K35" t="s">
+        <v>238</v>
+      </c>
+      <c r="L35" t="s">
+        <v>239</v>
+      </c>
+      <c r="M35" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>127</v>
+      </c>
+      <c r="G36" t="s">
+        <v>238</v>
+      </c>
+      <c r="H36" t="s">
+        <v>239</v>
+      </c>
+      <c r="I36" t="s">
+        <v>239</v>
+      </c>
+      <c r="J36" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>51</v>
+      </c>
+      <c r="F37" t="s">
+        <v>238</v>
+      </c>
+      <c r="G37" t="s">
+        <v>239</v>
+      </c>
+      <c r="H37" t="s">
+        <v>239</v>
+      </c>
+      <c r="I37" t="s">
+        <v>239</v>
+      </c>
+      <c r="J37" t="s">
+        <v>239</v>
+      </c>
+      <c r="K37" t="s">
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -9980,13 +10788,13 @@
         <v>251</v>
       </c>
       <c r="O1" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
       <c r="P1" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="Q1" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
@@ -10006,7 +10814,7 @@
         <v>237</v>
       </c>
       <c r="P2" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
     </row>
   </sheetData>
@@ -20955,7 +21763,7 @@
         <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="J5" t="s">
         <v>238</v>
@@ -20975,7 +21783,7 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="I6" t="s">
         <v>238</v>
@@ -21315,7 +22123,7 @@
         <v>46</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="H20" t="s">
         <v>238</v>
@@ -21338,7 +22146,7 @@
         <v>47</v>
       </c>
       <c r="B21" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="I21" t="s">
         <v>238</v>
@@ -21352,7 +22160,7 @@
         <v>48</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="G22" t="s">
         <v>238</v>
@@ -21476,7 +22284,7 @@
         <v>50</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>508</v>
+        <v>524</v>
       </c>
       <c r="J27" t="s">
         <v>238</v>
@@ -21492,8 +22300,8 @@
       <c r="A28" t="s">
         <v>51</v>
       </c>
-      <c r="B28" t="s">
-        <v>127</v>
+      <c r="B28" s="1" t="s">
+        <v>525</v>
       </c>
       <c r="I28" t="s">
         <v>238</v>
@@ -29610,7 +30418,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="G4" t="s">
         <v>238</v>
@@ -29624,7 +30432,7 @@
         <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="H5" t="s">
         <v>239</v>
@@ -29822,7 +30630,7 @@
         <v>60</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>515</v>
+        <v>527</v>
       </c>
       <c r="G14" t="s">
         <v>238</v>
@@ -30090,7 +30898,7 @@
         <v>70</v>
       </c>
       <c r="B26" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="C26" t="s">
         <v>239</v>
@@ -30135,6 +30943,9 @@
       <c r="A28" s="1" t="s">
         <v>72</v>
       </c>
+      <c r="B28" s="1" t="s">
+        <v>508</v>
+      </c>
       <c r="D28" t="s">
         <v>238</v>
       </c>
@@ -30166,6 +30977,9 @@
       <c r="A30" s="1" t="s">
         <v>74</v>
       </c>
+      <c r="B30" s="1" t="s">
+        <v>508</v>
+      </c>
       <c r="I30" t="s">
         <v>238</v>
       </c>
@@ -30251,7 +31065,7 @@
         <v>76</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>508</v>
+        <v>526</v>
       </c>
       <c r="C33" t="s">
         <v>239</v>
@@ -30300,7 +31114,7 @@
         <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C35" t="s">
         <v>239</v>
@@ -30320,7 +31134,7 @@
         <v>77</v>
       </c>
       <c r="B36" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="C36" t="s">
         <v>239</v>
@@ -30364,7 +31178,7 @@
         <v>78</v>
       </c>
       <c r="B37" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="C37" t="s">
         <v>239</v>
@@ -30967,8 +31781,8 @@
       <c r="A60" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B60" s="7" t="s">
-        <v>518</v>
+      <c r="B60" s="5" t="s">
+        <v>528</v>
       </c>
       <c r="I60" t="s">
         <v>238</v>
@@ -30987,7 +31801,7 @@
       <c r="A61" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B61" s="8"/>
+      <c r="B61" s="6"/>
       <c r="I61" t="s">
         <v>238</v>
       </c>
@@ -31048,8 +31862,8 @@
       <c r="A64" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B64" s="7" t="s">
-        <v>520</v>
+      <c r="B64" s="5" t="s">
+        <v>529</v>
       </c>
       <c r="F64" t="s">
         <v>238</v>
@@ -31068,7 +31882,7 @@
       <c r="A65" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B65" s="8"/>
+      <c r="B65" s="6"/>
       <c r="F65" t="s">
         <v>238</v>
       </c>
@@ -31101,7 +31915,7 @@
         <v>101</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="C67" t="s">
         <v>239</v>
@@ -31121,7 +31935,7 @@
         <v>46</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="C68" t="s">
         <v>239</v>
@@ -31153,7 +31967,7 @@
         <v>102</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="C69" t="s">
         <v>239</v>
@@ -31173,7 +31987,7 @@
         <v>103</v>
       </c>
       <c r="B70" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="C70" t="s">
         <v>239</v>
@@ -31222,7 +32036,7 @@
         <v>12</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="H72" t="s">
         <v>238</v>
@@ -31242,7 +32056,7 @@
         <v>31</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="K73" t="s">
         <v>238</v>
@@ -31259,7 +32073,7 @@
         <v>104</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="C74" t="s">
         <v>239</v>
@@ -38785,6 +39599,9 @@
       <c r="A3" s="1" t="s">
         <v>36</v>
       </c>
+      <c r="B3" s="1" t="s">
+        <v>508</v>
+      </c>
       <c r="C3" t="s">
         <v>338</v>
       </c>
@@ -38858,6 +39675,9 @@
       <c r="A5" s="1" t="s">
         <v>108</v>
       </c>
+      <c r="B5" s="1" t="s">
+        <v>508</v>
+      </c>
       <c r="I5" t="s">
         <v>238</v>
       </c>
@@ -38907,6 +39727,9 @@
       <c r="A7" s="1" t="s">
         <v>109</v>
       </c>
+      <c r="B7" s="1" t="s">
+        <v>508</v>
+      </c>
       <c r="I7" t="s">
         <v>238</v>
       </c>
@@ -38925,7 +39748,7 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="C8" t="s">
         <v>338</v>
@@ -39186,7 +40009,7 @@
         <v>112</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>508</v>
+        <v>530</v>
       </c>
       <c r="F17" t="s">
         <v>238</v>
@@ -39264,7 +40087,7 @@
         <v>27</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="H20" t="s">
         <v>238</v>
@@ -39284,7 +40107,7 @@
         <v>113</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="F21" t="s">
         <v>238</v>
@@ -39330,7 +40153,7 @@
         <v>114</v>
       </c>
       <c r="B23" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H23" t="s">
         <v>238</v>
@@ -39393,7 +40216,7 @@
         <v>116</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="F26" t="s">
         <v>238</v>
@@ -39454,7 +40277,7 @@
         <v>117</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="H28" t="s">
         <v>238</v>
@@ -39474,7 +40297,7 @@
         <v>118</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="C29" t="s">
         <v>338</v>
@@ -39500,7 +40323,7 @@
         <v>119</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="C30" t="s">
         <v>338</v>
@@ -39735,7 +40558,7 @@
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="H41" t="s">
         <v>238</v>

</xml_diff>

<commit_message>
Minor updates mapping to consistent fork ranger names.
</commit_message>
<xml_diff>
--- a/data/raw/State_Sources.xlsx
+++ b/data/raw/State_Sources.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chigham\Documents\forkranger-us-regions\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE2235EC-A946-43A7-9500-90553C2C30C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7948CA-DB90-4A67-813F-0520E598491F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{1A035CB0-260D-4ABF-9F3B-5033D39FF1A0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1A035CB0-260D-4ABF-9F3B-5033D39FF1A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Alabama" sheetId="1" r:id="rId1"/>
@@ -21875,7 +21875,7 @@
         <v>40</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="H10" t="s">
         <v>238</v>

</xml_diff>

<commit_message>
Added source links to states. Added data for South Carolina. Corrected a source download to reflect the right state.
</commit_message>
<xml_diff>
--- a/data/raw/State_Sources.xlsx
+++ b/data/raw/State_Sources.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chigham\Documents\forkranger-us-regions\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7948CA-DB90-4A67-813F-0520E598491F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719D5691-97E3-40AA-9D54-057DB7AD251E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1A035CB0-260D-4ABF-9F3B-5033D39FF1A0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="44" activeTab="45" xr2:uid="{1A035CB0-260D-4ABF-9F3B-5033D39FF1A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Alabama" sheetId="1" r:id="rId1"/>
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15179" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15550" uniqueCount="562">
   <si>
     <t>Greens (Collards, turnips, etc.)</t>
   </si>
@@ -1711,6 +1711,93 @@
   </si>
   <si>
     <t>Extended Season</t>
+  </si>
+  <si>
+    <t>https://www.vdacs.virginia.gov/pdf/producechart.pdf</t>
+  </si>
+  <si>
+    <t>https://vtfeed.org/sites/default/files/imce/uploads/Vermont%20Harvest%20Calendar.pdf</t>
+  </si>
+  <si>
+    <t>https://files.nc.gov/ncoshr/Wellness_AvailabilityChart.pdf</t>
+  </si>
+  <si>
+    <t>https://idahopreferred.com/products/</t>
+  </si>
+  <si>
+    <t>This source is specific to Missouri</t>
+  </si>
+  <si>
+    <t>https://agriculture.ny.gov/system/files/documents/2019/03/harvestchart2016english.pdf</t>
+  </si>
+  <si>
+    <t>https://www.ndda.nd.gov/sites/www/files/documents/files/Seasonal%20Eating%20Guide_v2.pdf</t>
+  </si>
+  <si>
+    <t>https://ofbf.org/about/farm-to-table/whats-in-season/</t>
+  </si>
+  <si>
+    <t>THIS NEEDS TO BE REDONE</t>
+  </si>
+  <si>
+    <t>https://okfarmtoschool.com/wp-content/uploads/harvest-calendar.pdf</t>
+  </si>
+  <si>
+    <t>https://www.pa.gov/content/dam/copapwp-pagov/en/pda/documents/business-industry/pa_preferred/documents/SeasonalCalendar-2022.pdf</t>
+  </si>
+  <si>
+    <t>https://mcs.com.pr/en/PDFs/Nutricion_Abundance_Calendar_ENG.pdf</t>
+  </si>
+  <si>
+    <t>https://www.sd.gov/wic?id=kb_article_view&amp;sysparm_article=KB0041262&amp;sys_kb_id=51fc2c0a8790c210ad0932e40cbb3548&amp;spa=1</t>
+  </si>
+  <si>
+    <t>QUESTIONABLE SOURCE</t>
+  </si>
+  <si>
+    <t>https://www.bristoltn.gov/708/Crops-in-Season</t>
+  </si>
+  <si>
+    <t>https://texasagriculture.gov/Portals/0/forms/MKT/TDA%20Produce%20Commodity%20Card.pdf</t>
+  </si>
+  <si>
+    <t>https://www.utahfarmbureau.org/Utah-Farm-Bureau/Food/Farm-Bureau-Farmers-Markets</t>
+  </si>
+  <si>
+    <t>OTHER SOURCES ARE AVAILABLE AND CAN BE ADDED</t>
+  </si>
+  <si>
+    <t>https://alabamafarmtoece.org/wp-content/uploads/2022/04/ALSeasonal-Produce-Guide.pdf</t>
+  </si>
+  <si>
+    <t>https://certifiedsc.com/where-to-buy-local/whats-in-season/</t>
+  </si>
+  <si>
+    <t>Beans (Snap, Pole, Variety)</t>
+  </si>
+  <si>
+    <t>Green Peanuts</t>
+  </si>
+  <si>
+    <t>Mixed Leafy Greens (collards, etc.)</t>
+  </si>
+  <si>
+    <t>Peas (Snap, Sugar)</t>
+  </si>
+  <si>
+    <t>Peppers (Variety)</t>
+  </si>
+  <si>
+    <t>Potatoes Red</t>
+  </si>
+  <si>
+    <t>Potatoes White</t>
+  </si>
+  <si>
+    <t>Sun Chokes</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -7687,7 +7774,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A04CE69-1813-41B0-90C3-EE7A4808F415}">
   <sheetPr codeName="Sheet14"/>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
@@ -7697,7 +7784,7 @@
     <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -7734,8 +7821,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -7764,7 +7854,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>53</v>
       </c>
@@ -7775,7 +7865,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -7786,7 +7876,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>221</v>
       </c>
@@ -7797,7 +7887,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>222</v>
       </c>
@@ -7811,7 +7901,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -7825,7 +7915,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -7842,7 +7932,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>135</v>
       </c>
@@ -7859,7 +7949,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -7873,7 +7963,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -7884,7 +7974,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -7901,7 +7991,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>54</v>
       </c>
@@ -7912,7 +8002,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -7926,7 +8016,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -7940,7 +8030,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>137</v>
       </c>
@@ -10741,10 +10831,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E70CA01-BAE2-4227-8730-A04965E99B41}">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>501</v>
       </c>
@@ -10796,8 +10886,11 @@
       <c r="Q1" t="s">
         <v>520</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="S1" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -20213,6 +20306,9 @@
       </c>
       <c r="M2" t="s">
         <v>237</v>
+      </c>
+      <c r="N2" t="s">
+        <v>537</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -27303,14 +27399,14 @@
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB9A47CA-EEF1-4151-A46A-9938347DBA49}">
   <sheetPr codeName="Sheet34"/>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:N53"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="13" width="17.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -27347,8 +27443,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -27389,7 +27488,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -27400,7 +27499,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -27414,7 +27513,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -27425,7 +27524,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -27436,7 +27535,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>326</v>
       </c>
@@ -27444,7 +27543,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>123</v>
       </c>
@@ -27458,7 +27557,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -27472,7 +27571,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>64</v>
       </c>
@@ -27498,7 +27597,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>65</v>
       </c>
@@ -27515,7 +27614,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>150</v>
       </c>
@@ -27526,7 +27625,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -27540,7 +27639,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -27551,7 +27650,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>127</v>
       </c>
@@ -27562,7 +27661,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -28435,7 +28534,7 @@
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B5F2BCB-E954-4FB3-9902-5D527AA48DE9}">
   <sheetPr codeName="Sheet35"/>
-  <dimension ref="A1:M59"/>
+  <dimension ref="A1:N59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.21875" bestFit="1" customWidth="1"/>
@@ -28443,7 +28542,7 @@
     <col min="4" max="13" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -28480,8 +28579,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -28507,7 +28609,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -28518,7 +28620,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -28538,7 +28640,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -28552,7 +28654,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -28566,7 +28668,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>339</v>
       </c>
@@ -28586,7 +28688,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -28597,7 +28699,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>340</v>
       </c>
@@ -28608,7 +28710,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -28637,7 +28739,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -28648,7 +28750,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -28665,7 +28767,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>298</v>
       </c>
@@ -28682,7 +28784,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>41</v>
       </c>
@@ -28723,7 +28825,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -28743,7 +28845,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -29544,7 +29646,7 @@
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A1634EA-A489-4A13-B66B-6FBA758233DF}">
   <sheetPr codeName="Sheet36"/>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:N49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.44140625" bestFit="1" customWidth="1"/>
@@ -29556,7 +29658,7 @@
     <col min="13" max="13" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -29593,8 +29695,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -29611,7 +29716,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>54</v>
       </c>
@@ -29622,7 +29727,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>348</v>
       </c>
@@ -29633,7 +29738,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>326</v>
       </c>
@@ -29644,7 +29749,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>123</v>
       </c>
@@ -29655,7 +29760,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>349</v>
       </c>
@@ -29666,7 +29771,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>65</v>
       </c>
@@ -29677,7 +29782,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -29691,7 +29796,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>48</v>
       </c>
@@ -29705,7 +29810,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -29716,7 +29821,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>71</v>
       </c>
@@ -29727,7 +29832,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -29741,7 +29846,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -29758,7 +29863,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -29778,7 +29883,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>37</v>
       </c>
@@ -32208,10 +32313,14 @@
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCC7FB74-2730-4C97-9F77-7A57F1B9797E}">
   <sheetPr codeName="Sheet37"/>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="6" max="10" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -32248,8 +32357,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -32265,8 +32377,11 @@
       <c r="L2" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N2" s="1" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -32286,7 +32401,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -32309,7 +32424,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -32326,7 +32441,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -32340,7 +32455,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>55</v>
       </c>
@@ -32360,7 +32475,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>230</v>
       </c>
@@ -32383,7 +32498,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -32400,7 +32515,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>270</v>
       </c>
@@ -32420,7 +32535,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>123</v>
       </c>
@@ -32434,7 +32549,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -32457,7 +32572,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -32477,7 +32592,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -32494,7 +32609,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>316</v>
       </c>
@@ -32517,7 +32632,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -32803,7 +32918,7 @@
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71A36A21-2118-4F7C-8C75-9D2A75AA3523}">
   <sheetPr codeName="Sheet38"/>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.21875" bestFit="1" customWidth="1"/>
@@ -32813,7 +32928,7 @@
     <col min="11" max="13" width="11.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -32850,8 +32965,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -32871,7 +32989,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -32885,7 +33003,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -32911,7 +33029,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -32925,7 +33043,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>351</v>
       </c>
@@ -32942,7 +33060,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -32953,7 +33071,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -32976,7 +33094,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -32999,7 +33117,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>136</v>
       </c>
@@ -33016,7 +33134,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -33039,7 +33157,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -33059,7 +33177,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -33079,7 +33197,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -33096,7 +33214,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>137</v>
       </c>
@@ -33116,7 +33234,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>111</v>
       </c>
@@ -33674,7 +33792,7 @@
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{679A2919-020B-4253-9BEF-E2E16A6FC39C}">
   <sheetPr codeName="Sheet40"/>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
@@ -33684,7 +33802,7 @@
     <col min="13" max="13" width="17.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -33721,8 +33839,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -33754,7 +33875,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -33762,7 +33883,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>111</v>
       </c>
@@ -33776,7 +33897,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -33790,7 +33911,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -33804,7 +33925,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -33818,7 +33939,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -33835,7 +33956,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -33852,7 +33973,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>136</v>
       </c>
@@ -33863,7 +33984,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -33886,7 +34007,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -33903,7 +34024,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>54</v>
       </c>
@@ -33914,7 +34035,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -33928,7 +34049,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -33942,7 +34063,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -34375,14 +34496,14 @@
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E81C2A9-D250-4D1C-9235-C36A4FD70631}">
   <sheetPr codeName="Sheet41"/>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
     <col min="2" max="13" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -34419,8 +34540,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>358</v>
       </c>
@@ -34461,7 +34585,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>178</v>
       </c>
@@ -34502,7 +34626,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>359</v>
       </c>
@@ -34522,7 +34646,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -34545,7 +34669,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>119</v>
       </c>
@@ -34571,7 +34695,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -34594,7 +34718,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>100</v>
       </c>
@@ -34635,7 +34759,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>360</v>
       </c>
@@ -34664,7 +34788,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>113</v>
       </c>
@@ -34690,7 +34814,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>361</v>
       </c>
@@ -34731,7 +34855,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>362</v>
       </c>
@@ -34757,7 +34881,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>170</v>
       </c>
@@ -34777,7 +34901,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>186</v>
       </c>
@@ -34818,7 +34942,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -34844,7 +34968,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>363</v>
       </c>
@@ -35810,10 +35934,13 @@
 <file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{787C0560-B6AC-43B7-9D40-0BAAE1936FD6}">
   <sheetPr codeName="Sheet43"/>
-  <dimension ref="B1:M1"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -35849,6 +35976,1170 @@
       </c>
       <c r="M1" t="s">
         <v>251</v>
+      </c>
+      <c r="N1" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" t="s">
+        <v>561</v>
+      </c>
+      <c r="K2" t="s">
+        <v>561</v>
+      </c>
+      <c r="L2" t="s">
+        <v>561</v>
+      </c>
+      <c r="M2" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s">
+        <v>561</v>
+      </c>
+      <c r="F3" t="s">
+        <v>561</v>
+      </c>
+      <c r="J3" t="s">
+        <v>561</v>
+      </c>
+      <c r="K3" t="s">
+        <v>561</v>
+      </c>
+      <c r="L3" t="s">
+        <v>561</v>
+      </c>
+      <c r="M3" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" t="s">
+        <v>561</v>
+      </c>
+      <c r="E4" t="s">
+        <v>561</v>
+      </c>
+      <c r="F4" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>553</v>
+      </c>
+      <c r="F5" t="s">
+        <v>561</v>
+      </c>
+      <c r="G5" t="s">
+        <v>561</v>
+      </c>
+      <c r="H5" t="s">
+        <v>561</v>
+      </c>
+      <c r="I5" t="s">
+        <v>561</v>
+      </c>
+      <c r="J5" t="s">
+        <v>561</v>
+      </c>
+      <c r="K5" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>561</v>
+      </c>
+      <c r="C6" t="s">
+        <v>561</v>
+      </c>
+      <c r="D6" t="s">
+        <v>561</v>
+      </c>
+      <c r="E6" t="s">
+        <v>561</v>
+      </c>
+      <c r="F6" t="s">
+        <v>561</v>
+      </c>
+      <c r="K6" t="s">
+        <v>561</v>
+      </c>
+      <c r="L6" t="s">
+        <v>561</v>
+      </c>
+      <c r="M6" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" t="s">
+        <v>561</v>
+      </c>
+      <c r="H7" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>561</v>
+      </c>
+      <c r="F8" t="s">
+        <v>561</v>
+      </c>
+      <c r="G8" t="s">
+        <v>561</v>
+      </c>
+      <c r="H8" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" t="s">
+        <v>561</v>
+      </c>
+      <c r="E9" t="s">
+        <v>561</v>
+      </c>
+      <c r="F9" t="s">
+        <v>561</v>
+      </c>
+      <c r="G9" t="s">
+        <v>561</v>
+      </c>
+      <c r="J9" t="s">
+        <v>561</v>
+      </c>
+      <c r="K9" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" t="s">
+        <v>561</v>
+      </c>
+      <c r="F10" t="s">
+        <v>561</v>
+      </c>
+      <c r="G10" t="s">
+        <v>561</v>
+      </c>
+      <c r="K10" t="s">
+        <v>561</v>
+      </c>
+      <c r="L10" t="s">
+        <v>561</v>
+      </c>
+      <c r="M10" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>109</v>
+      </c>
+      <c r="G11" t="s">
+        <v>561</v>
+      </c>
+      <c r="H11" t="s">
+        <v>561</v>
+      </c>
+      <c r="I11" t="s">
+        <v>561</v>
+      </c>
+      <c r="J11" t="s">
+        <v>561</v>
+      </c>
+      <c r="K11" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>561</v>
+      </c>
+      <c r="C12" t="s">
+        <v>561</v>
+      </c>
+      <c r="D12" t="s">
+        <v>561</v>
+      </c>
+      <c r="E12" t="s">
+        <v>561</v>
+      </c>
+      <c r="F12" t="s">
+        <v>561</v>
+      </c>
+      <c r="G12" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" t="s">
+        <v>561</v>
+      </c>
+      <c r="H13" t="s">
+        <v>561</v>
+      </c>
+      <c r="I13" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>561</v>
+      </c>
+      <c r="C14" t="s">
+        <v>561</v>
+      </c>
+      <c r="D14" t="s">
+        <v>561</v>
+      </c>
+      <c r="E14" t="s">
+        <v>561</v>
+      </c>
+      <c r="F14" t="s">
+        <v>561</v>
+      </c>
+      <c r="J14" t="s">
+        <v>561</v>
+      </c>
+      <c r="K14" t="s">
+        <v>561</v>
+      </c>
+      <c r="L14" t="s">
+        <v>561</v>
+      </c>
+      <c r="M14" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="F15" t="s">
+        <v>561</v>
+      </c>
+      <c r="L15" t="s">
+        <v>561</v>
+      </c>
+      <c r="M15" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" t="s">
+        <v>561</v>
+      </c>
+      <c r="C16" t="s">
+        <v>561</v>
+      </c>
+      <c r="D16" t="s">
+        <v>561</v>
+      </c>
+      <c r="E16" t="s">
+        <v>561</v>
+      </c>
+      <c r="F16" t="s">
+        <v>561</v>
+      </c>
+      <c r="G16" t="s">
+        <v>561</v>
+      </c>
+      <c r="H16" t="s">
+        <v>561</v>
+      </c>
+      <c r="I16" t="s">
+        <v>561</v>
+      </c>
+      <c r="J16" t="s">
+        <v>561</v>
+      </c>
+      <c r="K16" t="s">
+        <v>561</v>
+      </c>
+      <c r="L16" t="s">
+        <v>561</v>
+      </c>
+      <c r="M16" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" t="s">
+        <v>561</v>
+      </c>
+      <c r="G17" t="s">
+        <v>561</v>
+      </c>
+      <c r="H17" t="s">
+        <v>561</v>
+      </c>
+      <c r="J17" t="s">
+        <v>561</v>
+      </c>
+      <c r="K17" t="s">
+        <v>561</v>
+      </c>
+      <c r="L17" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>294</v>
+      </c>
+      <c r="G18" t="s">
+        <v>561</v>
+      </c>
+      <c r="H18" t="s">
+        <v>561</v>
+      </c>
+      <c r="I18" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" t="s">
+        <v>561</v>
+      </c>
+      <c r="H19" t="s">
+        <v>561</v>
+      </c>
+      <c r="I19" t="s">
+        <v>561</v>
+      </c>
+      <c r="L19" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>321</v>
+      </c>
+      <c r="E20" t="s">
+        <v>561</v>
+      </c>
+      <c r="F20" t="s">
+        <v>561</v>
+      </c>
+      <c r="G20" t="s">
+        <v>561</v>
+      </c>
+      <c r="K20" t="s">
+        <v>561</v>
+      </c>
+      <c r="L20" t="s">
+        <v>561</v>
+      </c>
+      <c r="M20" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+      <c r="I21" t="s">
+        <v>561</v>
+      </c>
+      <c r="J21" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>195</v>
+      </c>
+      <c r="C22" t="s">
+        <v>561</v>
+      </c>
+      <c r="D22" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>554</v>
+      </c>
+      <c r="H23" t="s">
+        <v>561</v>
+      </c>
+      <c r="I23" t="s">
+        <v>561</v>
+      </c>
+      <c r="J23" t="s">
+        <v>561</v>
+      </c>
+      <c r="K23" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" t="s">
+        <v>561</v>
+      </c>
+      <c r="C24" t="s">
+        <v>561</v>
+      </c>
+      <c r="D24" t="s">
+        <v>561</v>
+      </c>
+      <c r="E24" t="s">
+        <v>561</v>
+      </c>
+      <c r="F24" t="s">
+        <v>561</v>
+      </c>
+      <c r="G24" t="s">
+        <v>561</v>
+      </c>
+      <c r="H24" t="s">
+        <v>561</v>
+      </c>
+      <c r="I24" t="s">
+        <v>561</v>
+      </c>
+      <c r="J24" t="s">
+        <v>561</v>
+      </c>
+      <c r="K24" t="s">
+        <v>561</v>
+      </c>
+      <c r="L24" t="s">
+        <v>561</v>
+      </c>
+      <c r="M24" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>87</v>
+      </c>
+      <c r="D25" t="s">
+        <v>561</v>
+      </c>
+      <c r="E25" t="s">
+        <v>561</v>
+      </c>
+      <c r="F25" t="s">
+        <v>561</v>
+      </c>
+      <c r="G25" t="s">
+        <v>561</v>
+      </c>
+      <c r="J25" t="s">
+        <v>561</v>
+      </c>
+      <c r="K25" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" t="s">
+        <v>561</v>
+      </c>
+      <c r="D26" t="s">
+        <v>561</v>
+      </c>
+      <c r="E26" t="s">
+        <v>561</v>
+      </c>
+      <c r="F26" t="s">
+        <v>561</v>
+      </c>
+      <c r="K26" t="s">
+        <v>561</v>
+      </c>
+      <c r="L26" t="s">
+        <v>561</v>
+      </c>
+      <c r="M26" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" t="s">
+        <v>561</v>
+      </c>
+      <c r="C27" t="s">
+        <v>561</v>
+      </c>
+      <c r="D27" t="s">
+        <v>561</v>
+      </c>
+      <c r="E27" t="s">
+        <v>561</v>
+      </c>
+      <c r="F27" t="s">
+        <v>561</v>
+      </c>
+      <c r="G27" t="s">
+        <v>561</v>
+      </c>
+      <c r="H27" t="s">
+        <v>561</v>
+      </c>
+      <c r="I27" t="s">
+        <v>561</v>
+      </c>
+      <c r="J27" t="s">
+        <v>561</v>
+      </c>
+      <c r="K27" t="s">
+        <v>561</v>
+      </c>
+      <c r="L27" t="s">
+        <v>561</v>
+      </c>
+      <c r="M27" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>555</v>
+      </c>
+      <c r="B28" t="s">
+        <v>561</v>
+      </c>
+      <c r="C28" t="s">
+        <v>561</v>
+      </c>
+      <c r="D28" t="s">
+        <v>561</v>
+      </c>
+      <c r="E28" t="s">
+        <v>561</v>
+      </c>
+      <c r="F28" t="s">
+        <v>561</v>
+      </c>
+      <c r="J28" t="s">
+        <v>561</v>
+      </c>
+      <c r="K28" t="s">
+        <v>561</v>
+      </c>
+      <c r="L28" t="s">
+        <v>561</v>
+      </c>
+      <c r="M28" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>343</v>
+      </c>
+      <c r="I29" t="s">
+        <v>561</v>
+      </c>
+      <c r="J29" t="s">
+        <v>561</v>
+      </c>
+      <c r="K29" t="s">
+        <v>561</v>
+      </c>
+      <c r="L29" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>90</v>
+      </c>
+      <c r="M30" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>27</v>
+      </c>
+      <c r="G31" t="s">
+        <v>561</v>
+      </c>
+      <c r="H31" t="s">
+        <v>561</v>
+      </c>
+      <c r="I31" t="s">
+        <v>561</v>
+      </c>
+      <c r="J31" t="s">
+        <v>561</v>
+      </c>
+      <c r="K31" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>10</v>
+      </c>
+      <c r="B32" t="s">
+        <v>561</v>
+      </c>
+      <c r="C32" t="s">
+        <v>561</v>
+      </c>
+      <c r="D32" t="s">
+        <v>561</v>
+      </c>
+      <c r="E32" t="s">
+        <v>561</v>
+      </c>
+      <c r="F32" t="s">
+        <v>561</v>
+      </c>
+      <c r="G32" t="s">
+        <v>561</v>
+      </c>
+      <c r="H32" t="s">
+        <v>561</v>
+      </c>
+      <c r="I32" t="s">
+        <v>561</v>
+      </c>
+      <c r="J32" t="s">
+        <v>561</v>
+      </c>
+      <c r="K32" t="s">
+        <v>561</v>
+      </c>
+      <c r="L32" t="s">
+        <v>561</v>
+      </c>
+      <c r="M32" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>19</v>
+      </c>
+      <c r="F33" t="s">
+        <v>561</v>
+      </c>
+      <c r="G33" t="s">
+        <v>561</v>
+      </c>
+      <c r="H33" t="s">
+        <v>561</v>
+      </c>
+      <c r="I33" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>45</v>
+      </c>
+      <c r="E34" t="s">
+        <v>561</v>
+      </c>
+      <c r="F34" t="s">
+        <v>561</v>
+      </c>
+      <c r="G34" t="s">
+        <v>561</v>
+      </c>
+      <c r="H34" t="s">
+        <v>561</v>
+      </c>
+      <c r="I34" t="s">
+        <v>561</v>
+      </c>
+      <c r="J34" t="s">
+        <v>561</v>
+      </c>
+      <c r="K34" t="s">
+        <v>561</v>
+      </c>
+      <c r="L34" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>556</v>
+      </c>
+      <c r="E35" t="s">
+        <v>561</v>
+      </c>
+      <c r="F35" t="s">
+        <v>561</v>
+      </c>
+      <c r="G35" t="s">
+        <v>561</v>
+      </c>
+      <c r="H35" t="s">
+        <v>561</v>
+      </c>
+      <c r="I35" t="s">
+        <v>561</v>
+      </c>
+      <c r="J35" t="s">
+        <v>561</v>
+      </c>
+      <c r="K35" t="s">
+        <v>561</v>
+      </c>
+      <c r="L35" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>557</v>
+      </c>
+      <c r="G36" t="s">
+        <v>561</v>
+      </c>
+      <c r="H36" t="s">
+        <v>561</v>
+      </c>
+      <c r="I36" t="s">
+        <v>561</v>
+      </c>
+      <c r="J36" t="s">
+        <v>561</v>
+      </c>
+      <c r="K36" t="s">
+        <v>561</v>
+      </c>
+      <c r="L36" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>65</v>
+      </c>
+      <c r="G37" t="s">
+        <v>561</v>
+      </c>
+      <c r="H37" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>21</v>
+      </c>
+      <c r="I38" t="s">
+        <v>561</v>
+      </c>
+      <c r="J38" t="s">
+        <v>561</v>
+      </c>
+      <c r="K38" t="s">
+        <v>561</v>
+      </c>
+      <c r="L38" t="s">
+        <v>561</v>
+      </c>
+      <c r="M38" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>558</v>
+      </c>
+      <c r="D39" t="s">
+        <v>561</v>
+      </c>
+      <c r="E39" t="s">
+        <v>561</v>
+      </c>
+      <c r="F39" t="s">
+        <v>561</v>
+      </c>
+      <c r="G39" t="s">
+        <v>561</v>
+      </c>
+      <c r="H39" t="s">
+        <v>561</v>
+      </c>
+      <c r="I39" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>559</v>
+      </c>
+      <c r="D40" t="s">
+        <v>561</v>
+      </c>
+      <c r="E40" t="s">
+        <v>561</v>
+      </c>
+      <c r="F40" t="s">
+        <v>561</v>
+      </c>
+      <c r="G40" t="s">
+        <v>561</v>
+      </c>
+      <c r="H40" t="s">
+        <v>561</v>
+      </c>
+      <c r="I40" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>33</v>
+      </c>
+      <c r="J41" t="s">
+        <v>561</v>
+      </c>
+      <c r="K41" t="s">
+        <v>561</v>
+      </c>
+      <c r="L41" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>46</v>
+      </c>
+      <c r="C42" t="s">
+        <v>561</v>
+      </c>
+      <c r="D42" t="s">
+        <v>561</v>
+      </c>
+      <c r="E42" t="s">
+        <v>561</v>
+      </c>
+      <c r="F42" t="s">
+        <v>561</v>
+      </c>
+      <c r="G42" t="s">
+        <v>561</v>
+      </c>
+      <c r="J42" t="s">
+        <v>561</v>
+      </c>
+      <c r="K42" t="s">
+        <v>561</v>
+      </c>
+      <c r="L42" t="s">
+        <v>561</v>
+      </c>
+      <c r="M42" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>47</v>
+      </c>
+      <c r="G43" t="s">
+        <v>561</v>
+      </c>
+      <c r="H43" t="s">
+        <v>561</v>
+      </c>
+      <c r="I43" t="s">
+        <v>561</v>
+      </c>
+      <c r="J43" t="s">
+        <v>561</v>
+      </c>
+      <c r="K43" t="s">
+        <v>561</v>
+      </c>
+      <c r="L43" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>155</v>
+      </c>
+      <c r="B44" t="s">
+        <v>561</v>
+      </c>
+      <c r="C44" t="s">
+        <v>561</v>
+      </c>
+      <c r="D44" t="s">
+        <v>561</v>
+      </c>
+      <c r="E44" t="s">
+        <v>561</v>
+      </c>
+      <c r="F44" t="s">
+        <v>561</v>
+      </c>
+      <c r="K44" t="s">
+        <v>561</v>
+      </c>
+      <c r="L44" t="s">
+        <v>561</v>
+      </c>
+      <c r="M44" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>6</v>
+      </c>
+      <c r="E45" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>172</v>
+      </c>
+      <c r="F46" t="s">
+        <v>561</v>
+      </c>
+      <c r="G46" t="s">
+        <v>561</v>
+      </c>
+      <c r="H46" t="s">
+        <v>561</v>
+      </c>
+      <c r="I46" t="s">
+        <v>561</v>
+      </c>
+      <c r="J46" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>4</v>
+      </c>
+      <c r="D47" t="s">
+        <v>561</v>
+      </c>
+      <c r="E47" t="s">
+        <v>561</v>
+      </c>
+      <c r="F47" t="s">
+        <v>561</v>
+      </c>
+      <c r="G47" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>560</v>
+      </c>
+      <c r="L48" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>162</v>
+      </c>
+      <c r="F49" t="s">
+        <v>561</v>
+      </c>
+      <c r="G49" t="s">
+        <v>561</v>
+      </c>
+      <c r="H49" t="s">
+        <v>561</v>
+      </c>
+      <c r="I49" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>167</v>
+      </c>
+      <c r="I50" t="s">
+        <v>561</v>
+      </c>
+      <c r="J50" t="s">
+        <v>561</v>
+      </c>
+      <c r="K50" t="s">
+        <v>561</v>
+      </c>
+      <c r="L50" t="s">
+        <v>561</v>
+      </c>
+      <c r="M50" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>104</v>
+      </c>
+      <c r="D51" t="s">
+        <v>561</v>
+      </c>
+      <c r="E51" t="s">
+        <v>561</v>
+      </c>
+      <c r="F51" t="s">
+        <v>561</v>
+      </c>
+      <c r="G51" t="s">
+        <v>561</v>
+      </c>
+      <c r="J51" t="s">
+        <v>561</v>
+      </c>
+      <c r="K51" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>23</v>
+      </c>
+      <c r="G52" t="s">
+        <v>561</v>
+      </c>
+      <c r="H52" t="s">
+        <v>561</v>
+      </c>
+      <c r="J52" t="s">
+        <v>561</v>
+      </c>
+      <c r="K52" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>49</v>
+      </c>
+      <c r="B53" t="s">
+        <v>561</v>
+      </c>
+      <c r="C53" t="s">
+        <v>561</v>
+      </c>
+      <c r="D53" t="s">
+        <v>561</v>
+      </c>
+      <c r="E53" t="s">
+        <v>561</v>
+      </c>
+      <c r="F53" t="s">
+        <v>561</v>
+      </c>
+      <c r="K53" t="s">
+        <v>561</v>
+      </c>
+      <c r="L53" t="s">
+        <v>561</v>
+      </c>
+      <c r="M53" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>24</v>
+      </c>
+      <c r="G54" t="s">
+        <v>561</v>
+      </c>
+      <c r="H54" t="s">
+        <v>561</v>
+      </c>
+      <c r="I54" t="s">
+        <v>561</v>
+      </c>
+      <c r="J54" t="s">
+        <v>561</v>
+      </c>
+      <c r="K54" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>51</v>
+      </c>
+      <c r="F55" t="s">
+        <v>561</v>
+      </c>
+      <c r="G55" t="s">
+        <v>561</v>
+      </c>
+      <c r="H55" t="s">
+        <v>561</v>
+      </c>
+      <c r="I55" t="s">
+        <v>561</v>
+      </c>
+      <c r="J55" t="s">
+        <v>561</v>
       </c>
     </row>
   </sheetData>
@@ -35859,14 +37150,14 @@
 <file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2613B65B-C97D-4F7F-A93B-55F0E2809563}">
   <sheetPr codeName="Sheet44"/>
-  <dimension ref="A1:M62"/>
+  <dimension ref="A1:N62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="13" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -35903,8 +37194,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>71</v>
       </c>
@@ -35914,8 +37208,11 @@
       <c r="G2" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N2" s="1" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -35950,7 +37247,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -35970,7 +37267,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -35990,7 +37287,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -36019,7 +37316,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -36054,7 +37351,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -36095,7 +37392,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -36109,7 +37406,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>39</v>
       </c>
@@ -36150,7 +37447,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -36185,7 +37482,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -36196,7 +37493,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -36207,7 +37504,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -36218,7 +37515,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>137</v>
       </c>
@@ -36244,7 +37541,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>272</v>
       </c>
@@ -37282,14 +38579,14 @@
 <file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1842B056-2474-4B33-9255-1B707810B331}">
   <sheetPr codeName="Sheet45"/>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="13" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -37326,8 +38623,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -37350,7 +38650,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -37364,7 +38664,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -37387,7 +38687,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -37410,7 +38710,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -37433,7 +38733,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -37447,7 +38747,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -37479,7 +38779,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -37511,7 +38811,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -37534,7 +38834,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -37575,7 +38875,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -37589,7 +38889,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>54</v>
       </c>
@@ -37612,7 +38912,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>41</v>
       </c>
@@ -37644,7 +38944,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -37667,7 +38967,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -38359,13 +39659,13 @@
 <file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA657458-A606-4E65-963F-0E27322C62D8}">
   <sheetPr codeName="Sheet46"/>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -38402,8 +39702,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -38426,7 +39729,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -38452,7 +39755,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -38466,7 +39769,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -38480,7 +39783,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -38497,7 +39800,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>211</v>
       </c>
@@ -38514,7 +39817,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>383</v>
       </c>
@@ -38555,7 +39858,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>384</v>
       </c>
@@ -38575,7 +39878,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>385</v>
       </c>
@@ -38592,7 +39895,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -38612,7 +39915,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -38653,7 +39956,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -38676,7 +39979,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>39</v>
       </c>
@@ -38696,7 +39999,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -38728,7 +40031,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>81</v>
       </c>
@@ -40759,7 +42062,7 @@
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2773CF06-5366-4382-B358-E65FDF97334C}">
   <sheetPr codeName="Sheet47"/>
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -40769,7 +42072,7 @@
     <col min="13" max="13" width="17.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -40806,8 +42109,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -40832,8 +42138,11 @@
       <c r="M2" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N2" s="1" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>53</v>
       </c>
@@ -40844,7 +42153,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>70</v>
       </c>
@@ -40867,7 +42176,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>41</v>
       </c>
@@ -40890,7 +42199,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -40913,7 +42222,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>388</v>
       </c>
@@ -40936,7 +42245,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>311</v>
       </c>
@@ -40959,7 +42268,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>71</v>
       </c>
@@ -40970,7 +42279,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -40990,7 +42299,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>158</v>
       </c>
@@ -41004,7 +42313,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -41021,7 +42330,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -41038,7 +42347,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -41058,7 +42367,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>122</v>
       </c>
@@ -41072,7 +42381,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>38</v>
       </c>
@@ -41456,7 +42765,7 @@
 <file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447A2CF6-2296-4430-A13E-509B8B6085A0}">
   <sheetPr codeName="Sheet48"/>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.44140625" bestFit="1" customWidth="1"/>
@@ -41468,7 +42777,7 @@
     <col min="13" max="13" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -41505,8 +42814,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -41538,7 +42850,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -41549,7 +42861,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -41566,7 +42878,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -41598,7 +42910,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -41606,7 +42918,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -41620,7 +42932,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -41640,7 +42952,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -41657,7 +42969,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -41683,7 +42995,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -41718,7 +43030,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -41738,7 +43050,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>320</v>
       </c>
@@ -41758,7 +43070,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>39</v>
       </c>
@@ -41775,7 +43087,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -41786,7 +43098,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -42339,7 +43651,7 @@
 <file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6430A47B-DF13-4154-9DC7-5A6C5E0BF723}">
   <sheetPr codeName="Sheet49"/>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
@@ -42349,7 +43661,7 @@
     <col min="12" max="13" width="11.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>240</v>
       </c>
@@ -42386,8 +43698,11 @@
       <c r="M1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -42422,7 +43737,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>64</v>
       </c>
@@ -42439,7 +43754,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -42453,7 +43768,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -42479,7 +43794,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -42493,7 +43808,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -42507,7 +43822,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -42521,7 +43836,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -42544,7 +43859,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -42555,7 +43870,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>42</v>
       </c>
@@ -42575,7 +43890,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -42589,7 +43904,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>123</v>
       </c>
@@ -42603,7 +43918,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>111</v>
       </c>
@@ -42623,7 +43938,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>177</v>
       </c>
@@ -42649,7 +43964,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
Updated language in RI farm flavor data table.
</commit_message>
<xml_diff>
--- a/data/raw/State_Sources.xlsx
+++ b/data/raw/State_Sources.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chigham\Documents\forkranger-us-regions\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C0E12C7-7836-4EAC-B678-006C918C0197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{048CFF4E-AC90-44B5-97D6-9399DEF14893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="42" activeTab="44" xr2:uid="{1A035CB0-260D-4ABF-9F3B-5033D39FF1A0}"/>
   </bookViews>
@@ -36048,16 +36048,16 @@
         <v>28</v>
       </c>
       <c r="H2" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I2" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J2" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K2" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -36065,13 +36065,13 @@
         <v>71</v>
       </c>
       <c r="E3" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="F3" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="G3" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -36079,16 +36079,16 @@
         <v>36</v>
       </c>
       <c r="H4" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I4" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J4" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K4" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -36096,22 +36096,22 @@
         <v>8</v>
       </c>
       <c r="F5" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="G5" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="H5" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="I5" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J5" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K5" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -36119,10 +36119,10 @@
         <v>25</v>
       </c>
       <c r="H6" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I6" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -36130,16 +36130,16 @@
         <v>14</v>
       </c>
       <c r="H7" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I7" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J7" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K7" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -36147,22 +36147,22 @@
         <v>15</v>
       </c>
       <c r="G8" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="H8" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="I8" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J8" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K8" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="L8" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -36170,22 +36170,22 @@
         <v>9</v>
       </c>
       <c r="G9" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="H9" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="I9" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J9" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K9" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="L9" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -36193,16 +36193,16 @@
         <v>5</v>
       </c>
       <c r="J10" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="K10" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="L10" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="M10" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -36210,7 +36210,7 @@
         <v>54</v>
       </c>
       <c r="G11" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -36218,25 +36218,25 @@
         <v>230</v>
       </c>
       <c r="F12" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="G12" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="H12" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="I12" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J12" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K12" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="L12" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
@@ -36244,16 +36244,16 @@
         <v>42</v>
       </c>
       <c r="G13" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="H13" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="I13" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J13" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -36261,16 +36261,16 @@
         <v>18</v>
       </c>
       <c r="H14" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I14" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J14" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K14" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -36278,10 +36278,10 @@
         <v>123</v>
       </c>
       <c r="I15" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="J15" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -36289,16 +36289,16 @@
         <v>197</v>
       </c>
       <c r="H16" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I16" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J16" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K16" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
@@ -36306,13 +36306,13 @@
         <v>168</v>
       </c>
       <c r="H17" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I17" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J17" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
@@ -36320,16 +36320,16 @@
         <v>27</v>
       </c>
       <c r="H18" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I18" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J18" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K18" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
@@ -36337,16 +36337,16 @@
         <v>10</v>
       </c>
       <c r="G19" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="H19" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="I19" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J19" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
@@ -36354,13 +36354,13 @@
         <v>19</v>
       </c>
       <c r="H20" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I20" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J20" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
@@ -36368,10 +36368,10 @@
         <v>64</v>
       </c>
       <c r="I21" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="J21" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
@@ -36379,22 +36379,22 @@
         <v>45</v>
       </c>
       <c r="F22" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="G22" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="H22" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="I22" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J22" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K22" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
@@ -36402,19 +36402,19 @@
         <v>22</v>
       </c>
       <c r="H23" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I23" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J23" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K23" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="L23" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
@@ -36422,16 +36422,16 @@
         <v>21</v>
       </c>
       <c r="H24" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I24" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J24" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K24" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
@@ -36439,10 +36439,10 @@
         <v>33</v>
       </c>
       <c r="J25" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="K25" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
@@ -36450,16 +36450,16 @@
         <v>47</v>
       </c>
       <c r="H26" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I26" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J26" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K26" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
@@ -36467,16 +36467,16 @@
         <v>48</v>
       </c>
       <c r="F27" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="G27" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="H27" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="I27" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
@@ -36484,13 +36484,13 @@
         <v>234</v>
       </c>
       <c r="G28" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="H28" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="I28" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
@@ -36498,16 +36498,16 @@
         <v>170</v>
       </c>
       <c r="G29" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="H29" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="I29" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J29" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
@@ -36515,13 +36515,13 @@
         <v>6</v>
       </c>
       <c r="E30" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="F30" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="G30" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
@@ -36529,13 +36529,13 @@
         <v>4</v>
       </c>
       <c r="F31" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="G31" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="H31" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
@@ -36543,16 +36543,16 @@
         <v>162</v>
       </c>
       <c r="H32" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I32" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J32" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K32" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
@@ -36560,16 +36560,16 @@
         <v>23</v>
       </c>
       <c r="H33" t="s">
-        <v>560</v>
+        <v>238</v>
       </c>
       <c r="I33" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="J33" t="s">
-        <v>560</v>
+        <v>239</v>
       </c>
       <c r="K33" t="s">
-        <v>560</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>

</xml_diff>